<commit_message>
updated test case file
</commit_message>
<xml_diff>
--- a/src/test/resources/flipkart_test_cases.xlsx
+++ b/src/test/resources/flipkart_test_cases.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27830"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yashgupta02\eclipse-qa\exit-test-automation\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nagarro-my.sharepoint.com/personal/yash_gupta02_nagarro_com/Documents/Desktop/github Projects/exit-test-automation/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89F5778E-895D-4EC1-BC1A-E04E98EC6BDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{89F5778E-895D-4EC1-BC1A-E04E98EC6BDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DEFBCDC8-CB9B-4BCB-AC41-E0B2B6C8BB7E}"/>
   <bookViews>
     <workbookView xWindow="1416" yWindow="1332" windowWidth="19788" windowHeight="9852" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -778,7 +778,7 @@
         <v>66</v>
       </c>
       <c r="F3" t="s">
-        <v>47</v>
+        <v>100</v>
       </c>
       <c r="G3" t="s">
         <v>67</v>

</xml_diff>